<commit_message>
feat: self assesment score and some fixes
</commit_message>
<xml_diff>
--- a/docs/My_Professional_Reviews/UAS-5_Skor.xlsx
+++ b/docs/My_Professional_Reviews/UAS-5_Skor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github3\2025_KIPP\asesmen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\all-about-me\My_Professional_Reviews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04162E76-CA32-4FBF-9F98-5B5AB9101282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF624EE-6643-4DE0-8790-527A83ADDF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8AFE3614-8754-EB4D-B44F-1C12FCF6F8C2}"/>
   </bookViews>
   <sheets>
     <sheet name="UAS_1_My_Concepts" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
   <si>
     <t>ID</t>
   </si>
@@ -118,14 +118,24 @@
   <si>
     <t>UAS-1_Usefulness</t>
   </si>
+  <si>
+    <t>M. Abizzar Gamadrian</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -180,14 +190,15 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,15 +515,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73929F8-86DE-C24C-A270-AE251CD40D12}">
   <dimension ref="A1:AP82"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="2" customWidth="1"/>
-    <col min="3" max="42" width="18.6640625" style="2" customWidth="1"/>
-    <col min="43" max="16384" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="14.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.69921875" style="2" customWidth="1"/>
+    <col min="3" max="42" width="18.69921875" style="2" customWidth="1"/>
+    <col min="43" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +581,7 @@
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -600,10 +611,28 @@
       <c r="AK2" s="3"/>
       <c r="AP2" s="3"/>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.75">
-      <c r="G3" s="4" t="str">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>13523155</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ref="G3:G66" si="0">IF(COUNT(C3:F3)=0,"",AVERAGE(C3:F3))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
@@ -613,7 +642,7 @@
       <c r="AK3" s="4"/>
       <c r="AP3" s="4"/>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -626,7 +655,7 @@
       <c r="AK4" s="4"/>
       <c r="AP4" s="4"/>
     </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G5" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -639,7 +668,7 @@
       <c r="AK5" s="4"/>
       <c r="AP5" s="4"/>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G6" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -652,7 +681,7 @@
       <c r="AK6" s="4"/>
       <c r="AP6" s="4"/>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G7" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -665,7 +694,7 @@
       <c r="AK7" s="4"/>
       <c r="AP7" s="4"/>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G8" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -678,7 +707,7 @@
       <c r="AK8" s="4"/>
       <c r="AP8" s="4"/>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G9" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -691,7 +720,7 @@
       <c r="AK9" s="4"/>
       <c r="AP9" s="4"/>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G10" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -704,7 +733,7 @@
       <c r="AK10" s="4"/>
       <c r="AP10" s="4"/>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G11" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -717,7 +746,7 @@
       <c r="AK11" s="4"/>
       <c r="AP11" s="4"/>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G12" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -730,7 +759,7 @@
       <c r="AK12" s="4"/>
       <c r="AP12" s="4"/>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G13" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -743,7 +772,7 @@
       <c r="AK13" s="4"/>
       <c r="AP13" s="4"/>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G14" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -756,7 +785,7 @@
       <c r="AK14" s="4"/>
       <c r="AP14" s="4"/>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G15" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -769,7 +798,7 @@
       <c r="AK15" s="4"/>
       <c r="AP15" s="4"/>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G16" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -782,7 +811,7 @@
       <c r="AK16" s="4"/>
       <c r="AP16" s="4"/>
     </row>
-    <row r="17" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="17" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G17" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -795,7 +824,7 @@
       <c r="AK17" s="4"/>
       <c r="AP17" s="4"/>
     </row>
-    <row r="18" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="18" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G18" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -808,7 +837,7 @@
       <c r="AK18" s="4"/>
       <c r="AP18" s="4"/>
     </row>
-    <row r="19" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="19" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G19" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -821,7 +850,7 @@
       <c r="AK19" s="4"/>
       <c r="AP19" s="4"/>
     </row>
-    <row r="20" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="20" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G20" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -834,7 +863,7 @@
       <c r="AK20" s="4"/>
       <c r="AP20" s="4"/>
     </row>
-    <row r="21" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="21" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G21" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -847,7 +876,7 @@
       <c r="AK21" s="4"/>
       <c r="AP21" s="4"/>
     </row>
-    <row r="22" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="22" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G22" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -860,7 +889,7 @@
       <c r="AK22" s="4"/>
       <c r="AP22" s="4"/>
     </row>
-    <row r="23" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="23" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G23" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -873,7 +902,7 @@
       <c r="AK23" s="4"/>
       <c r="AP23" s="4"/>
     </row>
-    <row r="24" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="24" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G24" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -886,7 +915,7 @@
       <c r="AK24" s="4"/>
       <c r="AP24" s="4"/>
     </row>
-    <row r="25" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="25" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G25" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -899,7 +928,7 @@
       <c r="AK25" s="4"/>
       <c r="AP25" s="4"/>
     </row>
-    <row r="26" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="26" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G26" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -912,7 +941,7 @@
       <c r="AK26" s="4"/>
       <c r="AP26" s="4"/>
     </row>
-    <row r="27" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="27" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G27" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -925,7 +954,7 @@
       <c r="AK27" s="4"/>
       <c r="AP27" s="4"/>
     </row>
-    <row r="28" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="28" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G28" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -938,7 +967,7 @@
       <c r="AK28" s="4"/>
       <c r="AP28" s="4"/>
     </row>
-    <row r="29" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="29" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G29" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -951,7 +980,7 @@
       <c r="AK29" s="4"/>
       <c r="AP29" s="4"/>
     </row>
-    <row r="30" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="30" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G30" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -964,7 +993,7 @@
       <c r="AK30" s="4"/>
       <c r="AP30" s="4"/>
     </row>
-    <row r="31" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="31" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G31" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -977,7 +1006,7 @@
       <c r="AK31" s="4"/>
       <c r="AP31" s="4"/>
     </row>
-    <row r="32" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="32" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G32" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -990,7 +1019,7 @@
       <c r="AK32" s="4"/>
       <c r="AP32" s="4"/>
     </row>
-    <row r="33" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="33" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G33" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1003,7 +1032,7 @@
       <c r="AK33" s="4"/>
       <c r="AP33" s="4"/>
     </row>
-    <row r="34" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="34" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G34" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1016,7 +1045,7 @@
       <c r="AK34" s="4"/>
       <c r="AP34" s="4"/>
     </row>
-    <row r="35" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="35" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G35" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1029,7 +1058,7 @@
       <c r="AK35" s="4"/>
       <c r="AP35" s="4"/>
     </row>
-    <row r="36" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="36" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G36" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1042,7 +1071,7 @@
       <c r="AK36" s="4"/>
       <c r="AP36" s="4"/>
     </row>
-    <row r="37" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="37" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G37" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1055,7 +1084,7 @@
       <c r="AK37" s="4"/>
       <c r="AP37" s="4"/>
     </row>
-    <row r="38" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="38" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G38" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1068,7 +1097,7 @@
       <c r="AK38" s="4"/>
       <c r="AP38" s="4"/>
     </row>
-    <row r="39" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="39" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G39" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1081,7 +1110,7 @@
       <c r="AK39" s="4"/>
       <c r="AP39" s="4"/>
     </row>
-    <row r="40" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="40" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G40" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1094,7 +1123,7 @@
       <c r="AK40" s="4"/>
       <c r="AP40" s="4"/>
     </row>
-    <row r="41" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="41" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G41" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1107,7 +1136,7 @@
       <c r="AK41" s="4"/>
       <c r="AP41" s="4"/>
     </row>
-    <row r="42" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="42" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G42" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1120,7 +1149,7 @@
       <c r="AK42" s="4"/>
       <c r="AP42" s="4"/>
     </row>
-    <row r="43" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="43" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G43" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1133,7 +1162,7 @@
       <c r="AK43" s="4"/>
       <c r="AP43" s="4"/>
     </row>
-    <row r="44" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="44" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G44" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1146,7 +1175,7 @@
       <c r="AK44" s="4"/>
       <c r="AP44" s="4"/>
     </row>
-    <row r="45" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="45" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G45" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1159,7 +1188,7 @@
       <c r="AK45" s="4"/>
       <c r="AP45" s="4"/>
     </row>
-    <row r="46" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="46" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G46" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1172,7 +1201,7 @@
       <c r="AK46" s="4"/>
       <c r="AP46" s="4"/>
     </row>
-    <row r="47" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="47" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G47" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1185,7 +1214,7 @@
       <c r="AK47" s="4"/>
       <c r="AP47" s="4"/>
     </row>
-    <row r="48" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="48" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G48" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1198,7 +1227,7 @@
       <c r="AK48" s="4"/>
       <c r="AP48" s="4"/>
     </row>
-    <row r="49" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="49" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G49" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1211,7 +1240,7 @@
       <c r="AK49" s="4"/>
       <c r="AP49" s="4"/>
     </row>
-    <row r="50" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="50" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G50" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1224,7 +1253,7 @@
       <c r="AK50" s="4"/>
       <c r="AP50" s="4"/>
     </row>
-    <row r="51" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="51" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G51" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1237,7 +1266,7 @@
       <c r="AK51" s="4"/>
       <c r="AP51" s="4"/>
     </row>
-    <row r="52" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="52" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G52" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1250,7 +1279,7 @@
       <c r="AK52" s="4"/>
       <c r="AP52" s="4"/>
     </row>
-    <row r="53" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="53" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G53" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1263,7 +1292,7 @@
       <c r="AK53" s="4"/>
       <c r="AP53" s="4"/>
     </row>
-    <row r="54" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="54" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G54" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1276,7 +1305,7 @@
       <c r="AK54" s="4"/>
       <c r="AP54" s="4"/>
     </row>
-    <row r="55" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="55" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G55" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1289,7 +1318,7 @@
       <c r="AK55" s="4"/>
       <c r="AP55" s="4"/>
     </row>
-    <row r="56" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="56" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G56" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1302,7 +1331,7 @@
       <c r="AK56" s="4"/>
       <c r="AP56" s="4"/>
     </row>
-    <row r="57" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="57" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G57" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1315,7 +1344,7 @@
       <c r="AK57" s="4"/>
       <c r="AP57" s="4"/>
     </row>
-    <row r="58" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="58" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G58" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1328,7 +1357,7 @@
       <c r="AK58" s="4"/>
       <c r="AP58" s="4"/>
     </row>
-    <row r="59" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="59" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G59" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1341,7 +1370,7 @@
       <c r="AK59" s="4"/>
       <c r="AP59" s="4"/>
     </row>
-    <row r="60" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="60" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G60" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1354,7 +1383,7 @@
       <c r="AK60" s="4"/>
       <c r="AP60" s="4"/>
     </row>
-    <row r="61" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="61" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G61" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1367,7 +1396,7 @@
       <c r="AK61" s="4"/>
       <c r="AP61" s="4"/>
     </row>
-    <row r="62" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="62" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G62" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1380,7 +1409,7 @@
       <c r="AK62" s="4"/>
       <c r="AP62" s="4"/>
     </row>
-    <row r="63" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="63" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G63" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1393,7 +1422,7 @@
       <c r="AK63" s="4"/>
       <c r="AP63" s="4"/>
     </row>
-    <row r="64" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="64" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G64" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1406,7 +1435,7 @@
       <c r="AK64" s="4"/>
       <c r="AP64" s="4"/>
     </row>
-    <row r="65" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="65" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G65" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1419,7 +1448,7 @@
       <c r="AK65" s="4"/>
       <c r="AP65" s="4"/>
     </row>
-    <row r="66" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="66" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G66" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1432,7 +1461,7 @@
       <c r="AK66" s="4"/>
       <c r="AP66" s="4"/>
     </row>
-    <row r="67" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="67" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G67" s="4" t="str">
         <f t="shared" ref="G67:G82" si="1">IF(COUNT(C67:F67)=0,"",AVERAGE(C67:F67))</f>
         <v/>
@@ -1445,7 +1474,7 @@
       <c r="AK67" s="4"/>
       <c r="AP67" s="4"/>
     </row>
-    <row r="68" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="68" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G68" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1458,7 +1487,7 @@
       <c r="AK68" s="4"/>
       <c r="AP68" s="4"/>
     </row>
-    <row r="69" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="69" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G69" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1471,7 +1500,7 @@
       <c r="AK69" s="4"/>
       <c r="AP69" s="4"/>
     </row>
-    <row r="70" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="70" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G70" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1484,7 +1513,7 @@
       <c r="AK70" s="4"/>
       <c r="AP70" s="4"/>
     </row>
-    <row r="71" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="71" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G71" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1497,7 +1526,7 @@
       <c r="AK71" s="4"/>
       <c r="AP71" s="4"/>
     </row>
-    <row r="72" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="72" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G72" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1510,7 +1539,7 @@
       <c r="AK72" s="4"/>
       <c r="AP72" s="4"/>
     </row>
-    <row r="73" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="73" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G73" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1523,7 +1552,7 @@
       <c r="AK73" s="4"/>
       <c r="AP73" s="4"/>
     </row>
-    <row r="74" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="74" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G74" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1536,7 +1565,7 @@
       <c r="AK74" s="4"/>
       <c r="AP74" s="4"/>
     </row>
-    <row r="75" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="75" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G75" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1549,7 +1578,7 @@
       <c r="AK75" s="4"/>
       <c r="AP75" s="4"/>
     </row>
-    <row r="76" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="76" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G76" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1562,7 +1591,7 @@
       <c r="AK76" s="4"/>
       <c r="AP76" s="4"/>
     </row>
-    <row r="77" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="77" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G77" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1575,7 +1604,7 @@
       <c r="AK77" s="4"/>
       <c r="AP77" s="4"/>
     </row>
-    <row r="78" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="78" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G78" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1588,7 +1617,7 @@
       <c r="AK78" s="4"/>
       <c r="AP78" s="4"/>
     </row>
-    <row r="79" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="79" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G79" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1601,7 +1630,7 @@
       <c r="AK79" s="4"/>
       <c r="AP79" s="4"/>
     </row>
-    <row r="80" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="80" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G80" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1614,7 +1643,7 @@
       <c r="AK80" s="4"/>
       <c r="AP80" s="4"/>
     </row>
-    <row r="81" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="81" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G81" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1627,7 +1656,7 @@
       <c r="AK81" s="4"/>
       <c r="AP81" s="4"/>
     </row>
-    <row r="82" spans="7:42" x14ac:dyDescent="0.75">
+    <row r="82" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G82" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -1654,15 +1683,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3204561E-E5BB-0640-805F-3DEAFF53B8FF}">
   <dimension ref="A1:AP82"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="2" customWidth="1"/>
-    <col min="3" max="42" width="18.6640625" style="2" customWidth="1"/>
-    <col min="43" max="16384" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="14.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.69921875" style="2" customWidth="1"/>
+    <col min="3" max="42" width="18.69921875" style="2" customWidth="1"/>
+    <col min="43" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1720,7 +1749,7 @@
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
     </row>
-    <row r="2" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -1750,10 +1779,28 @@
       <c r="AK2" s="3"/>
       <c r="AP2" s="3"/>
     </row>
-    <row r="3" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
-      <c r="G3" s="4" t="str">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>13523155</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ref="G3:G66" si="0">IF(COUNT(C3:F3)=0,"",AVERAGE(C3:F3))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
@@ -1763,7 +1810,7 @@
       <c r="AK3" s="4"/>
       <c r="AP3" s="4"/>
     </row>
-    <row r="4" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1776,7 +1823,7 @@
       <c r="AK4" s="4"/>
       <c r="AP4" s="4"/>
     </row>
-    <row r="5" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G5" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1789,7 +1836,7 @@
       <c r="AK5" s="4"/>
       <c r="AP5" s="4"/>
     </row>
-    <row r="6" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G6" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1802,7 +1849,7 @@
       <c r="AK6" s="4"/>
       <c r="AP6" s="4"/>
     </row>
-    <row r="7" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G7" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1815,7 +1862,7 @@
       <c r="AK7" s="4"/>
       <c r="AP7" s="4"/>
     </row>
-    <row r="8" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G8" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1828,7 +1875,7 @@
       <c r="AK8" s="4"/>
       <c r="AP8" s="4"/>
     </row>
-    <row r="9" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G9" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1841,7 +1888,7 @@
       <c r="AK9" s="4"/>
       <c r="AP9" s="4"/>
     </row>
-    <row r="10" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G10" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1854,7 +1901,7 @@
       <c r="AK10" s="4"/>
       <c r="AP10" s="4"/>
     </row>
-    <row r="11" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G11" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1867,7 +1914,7 @@
       <c r="AK11" s="4"/>
       <c r="AP11" s="4"/>
     </row>
-    <row r="12" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G12" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1880,7 +1927,7 @@
       <c r="AK12" s="4"/>
       <c r="AP12" s="4"/>
     </row>
-    <row r="13" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G13" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1893,7 +1940,7 @@
       <c r="AK13" s="4"/>
       <c r="AP13" s="4"/>
     </row>
-    <row r="14" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G14" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1906,7 +1953,7 @@
       <c r="AK14" s="4"/>
       <c r="AP14" s="4"/>
     </row>
-    <row r="15" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G15" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1919,7 +1966,7 @@
       <c r="AK15" s="4"/>
       <c r="AP15" s="4"/>
     </row>
-    <row r="16" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G16" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1932,7 +1979,7 @@
       <c r="AK16" s="4"/>
       <c r="AP16" s="4"/>
     </row>
-    <row r="17" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="17" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G17" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1945,7 +1992,7 @@
       <c r="AK17" s="4"/>
       <c r="AP17" s="4"/>
     </row>
-    <row r="18" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="18" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G18" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1958,7 +2005,7 @@
       <c r="AK18" s="4"/>
       <c r="AP18" s="4"/>
     </row>
-    <row r="19" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="19" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G19" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1971,7 +2018,7 @@
       <c r="AK19" s="4"/>
       <c r="AP19" s="4"/>
     </row>
-    <row r="20" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="20" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G20" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1984,7 +2031,7 @@
       <c r="AK20" s="4"/>
       <c r="AP20" s="4"/>
     </row>
-    <row r="21" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="21" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G21" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1997,7 +2044,7 @@
       <c r="AK21" s="4"/>
       <c r="AP21" s="4"/>
     </row>
-    <row r="22" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="22" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G22" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2010,7 +2057,7 @@
       <c r="AK22" s="4"/>
       <c r="AP22" s="4"/>
     </row>
-    <row r="23" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="23" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G23" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2023,7 +2070,7 @@
       <c r="AK23" s="4"/>
       <c r="AP23" s="4"/>
     </row>
-    <row r="24" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="24" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G24" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2036,7 +2083,7 @@
       <c r="AK24" s="4"/>
       <c r="AP24" s="4"/>
     </row>
-    <row r="25" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="25" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G25" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2049,7 +2096,7 @@
       <c r="AK25" s="4"/>
       <c r="AP25" s="4"/>
     </row>
-    <row r="26" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="26" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G26" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2062,7 +2109,7 @@
       <c r="AK26" s="4"/>
       <c r="AP26" s="4"/>
     </row>
-    <row r="27" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="27" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G27" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2075,7 +2122,7 @@
       <c r="AK27" s="4"/>
       <c r="AP27" s="4"/>
     </row>
-    <row r="28" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="28" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G28" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2088,7 +2135,7 @@
       <c r="AK28" s="4"/>
       <c r="AP28" s="4"/>
     </row>
-    <row r="29" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="29" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G29" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2101,7 +2148,7 @@
       <c r="AK29" s="4"/>
       <c r="AP29" s="4"/>
     </row>
-    <row r="30" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="30" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G30" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2114,7 +2161,7 @@
       <c r="AK30" s="4"/>
       <c r="AP30" s="4"/>
     </row>
-    <row r="31" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="31" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G31" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2127,7 +2174,7 @@
       <c r="AK31" s="4"/>
       <c r="AP31" s="4"/>
     </row>
-    <row r="32" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="32" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G32" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2140,7 +2187,7 @@
       <c r="AK32" s="4"/>
       <c r="AP32" s="4"/>
     </row>
-    <row r="33" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="33" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G33" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2153,7 +2200,7 @@
       <c r="AK33" s="4"/>
       <c r="AP33" s="4"/>
     </row>
-    <row r="34" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="34" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G34" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2166,7 +2213,7 @@
       <c r="AK34" s="4"/>
       <c r="AP34" s="4"/>
     </row>
-    <row r="35" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="35" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G35" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2179,7 +2226,7 @@
       <c r="AK35" s="4"/>
       <c r="AP35" s="4"/>
     </row>
-    <row r="36" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="36" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G36" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2192,7 +2239,7 @@
       <c r="AK36" s="4"/>
       <c r="AP36" s="4"/>
     </row>
-    <row r="37" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="37" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G37" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2205,7 +2252,7 @@
       <c r="AK37" s="4"/>
       <c r="AP37" s="4"/>
     </row>
-    <row r="38" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="38" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G38" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2218,7 +2265,7 @@
       <c r="AK38" s="4"/>
       <c r="AP38" s="4"/>
     </row>
-    <row r="39" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="39" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G39" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2231,7 +2278,7 @@
       <c r="AK39" s="4"/>
       <c r="AP39" s="4"/>
     </row>
-    <row r="40" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="40" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G40" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2244,7 +2291,7 @@
       <c r="AK40" s="4"/>
       <c r="AP40" s="4"/>
     </row>
-    <row r="41" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="41" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G41" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2257,7 +2304,7 @@
       <c r="AK41" s="4"/>
       <c r="AP41" s="4"/>
     </row>
-    <row r="42" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="42" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G42" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2270,7 +2317,7 @@
       <c r="AK42" s="4"/>
       <c r="AP42" s="4"/>
     </row>
-    <row r="43" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="43" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G43" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2283,7 +2330,7 @@
       <c r="AK43" s="4"/>
       <c r="AP43" s="4"/>
     </row>
-    <row r="44" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="44" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G44" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2296,7 +2343,7 @@
       <c r="AK44" s="4"/>
       <c r="AP44" s="4"/>
     </row>
-    <row r="45" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="45" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G45" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2309,7 +2356,7 @@
       <c r="AK45" s="4"/>
       <c r="AP45" s="4"/>
     </row>
-    <row r="46" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="46" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G46" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2322,7 +2369,7 @@
       <c r="AK46" s="4"/>
       <c r="AP46" s="4"/>
     </row>
-    <row r="47" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="47" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G47" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2335,7 +2382,7 @@
       <c r="AK47" s="4"/>
       <c r="AP47" s="4"/>
     </row>
-    <row r="48" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="48" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G48" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2348,7 +2395,7 @@
       <c r="AK48" s="4"/>
       <c r="AP48" s="4"/>
     </row>
-    <row r="49" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="49" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G49" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2361,7 +2408,7 @@
       <c r="AK49" s="4"/>
       <c r="AP49" s="4"/>
     </row>
-    <row r="50" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="50" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G50" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2374,7 +2421,7 @@
       <c r="AK50" s="4"/>
       <c r="AP50" s="4"/>
     </row>
-    <row r="51" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="51" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G51" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2387,7 +2434,7 @@
       <c r="AK51" s="4"/>
       <c r="AP51" s="4"/>
     </row>
-    <row r="52" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="52" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G52" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2400,7 +2447,7 @@
       <c r="AK52" s="4"/>
       <c r="AP52" s="4"/>
     </row>
-    <row r="53" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="53" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G53" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2413,7 +2460,7 @@
       <c r="AK53" s="4"/>
       <c r="AP53" s="4"/>
     </row>
-    <row r="54" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="54" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G54" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2426,7 +2473,7 @@
       <c r="AK54" s="4"/>
       <c r="AP54" s="4"/>
     </row>
-    <row r="55" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="55" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G55" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2439,7 +2486,7 @@
       <c r="AK55" s="4"/>
       <c r="AP55" s="4"/>
     </row>
-    <row r="56" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="56" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G56" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2452,7 +2499,7 @@
       <c r="AK56" s="4"/>
       <c r="AP56" s="4"/>
     </row>
-    <row r="57" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="57" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G57" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2465,7 +2512,7 @@
       <c r="AK57" s="4"/>
       <c r="AP57" s="4"/>
     </row>
-    <row r="58" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="58" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G58" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2478,7 +2525,7 @@
       <c r="AK58" s="4"/>
       <c r="AP58" s="4"/>
     </row>
-    <row r="59" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="59" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G59" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2491,7 +2538,7 @@
       <c r="AK59" s="4"/>
       <c r="AP59" s="4"/>
     </row>
-    <row r="60" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="60" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G60" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2504,7 +2551,7 @@
       <c r="AK60" s="4"/>
       <c r="AP60" s="4"/>
     </row>
-    <row r="61" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="61" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G61" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2517,7 +2564,7 @@
       <c r="AK61" s="4"/>
       <c r="AP61" s="4"/>
     </row>
-    <row r="62" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="62" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G62" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2530,7 +2577,7 @@
       <c r="AK62" s="4"/>
       <c r="AP62" s="4"/>
     </row>
-    <row r="63" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="63" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G63" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2543,7 +2590,7 @@
       <c r="AK63" s="4"/>
       <c r="AP63" s="4"/>
     </row>
-    <row r="64" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="64" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G64" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2556,7 +2603,7 @@
       <c r="AK64" s="4"/>
       <c r="AP64" s="4"/>
     </row>
-    <row r="65" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="65" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G65" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2569,7 +2616,7 @@
       <c r="AK65" s="4"/>
       <c r="AP65" s="4"/>
     </row>
-    <row r="66" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="66" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G66" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2582,7 +2629,7 @@
       <c r="AK66" s="4"/>
       <c r="AP66" s="4"/>
     </row>
-    <row r="67" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="67" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G67" s="4" t="str">
         <f t="shared" ref="G67:G82" si="1">IF(COUNT(C67:F67)=0,"",AVERAGE(C67:F67))</f>
         <v/>
@@ -2595,7 +2642,7 @@
       <c r="AK67" s="4"/>
       <c r="AP67" s="4"/>
     </row>
-    <row r="68" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="68" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G68" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2608,7 +2655,7 @@
       <c r="AK68" s="4"/>
       <c r="AP68" s="4"/>
     </row>
-    <row r="69" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="69" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G69" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2621,7 +2668,7 @@
       <c r="AK69" s="4"/>
       <c r="AP69" s="4"/>
     </row>
-    <row r="70" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="70" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G70" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2634,7 +2681,7 @@
       <c r="AK70" s="4"/>
       <c r="AP70" s="4"/>
     </row>
-    <row r="71" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="71" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G71" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2647,7 +2694,7 @@
       <c r="AK71" s="4"/>
       <c r="AP71" s="4"/>
     </row>
-    <row r="72" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="72" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G72" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2660,7 +2707,7 @@
       <c r="AK72" s="4"/>
       <c r="AP72" s="4"/>
     </row>
-    <row r="73" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="73" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G73" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2673,7 +2720,7 @@
       <c r="AK73" s="4"/>
       <c r="AP73" s="4"/>
     </row>
-    <row r="74" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="74" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G74" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2686,7 +2733,7 @@
       <c r="AK74" s="4"/>
       <c r="AP74" s="4"/>
     </row>
-    <row r="75" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="75" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G75" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2699,7 +2746,7 @@
       <c r="AK75" s="4"/>
       <c r="AP75" s="4"/>
     </row>
-    <row r="76" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="76" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G76" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2712,7 +2759,7 @@
       <c r="AK76" s="4"/>
       <c r="AP76" s="4"/>
     </row>
-    <row r="77" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="77" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G77" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2725,7 +2772,7 @@
       <c r="AK77" s="4"/>
       <c r="AP77" s="4"/>
     </row>
-    <row r="78" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="78" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G78" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2738,7 +2785,7 @@
       <c r="AK78" s="4"/>
       <c r="AP78" s="4"/>
     </row>
-    <row r="79" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="79" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G79" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2751,7 +2798,7 @@
       <c r="AK79" s="4"/>
       <c r="AP79" s="4"/>
     </row>
-    <row r="80" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="80" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G80" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2764,7 +2811,7 @@
       <c r="AK80" s="4"/>
       <c r="AP80" s="4"/>
     </row>
-    <row r="81" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="81" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G81" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2777,7 +2824,7 @@
       <c r="AK81" s="4"/>
       <c r="AP81" s="4"/>
     </row>
-    <row r="82" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="82" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G82" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2804,15 +2851,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118772BA-2C36-4B0B-9DD9-177CEE93B495}">
   <dimension ref="A1:AP82"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="2" customWidth="1"/>
-    <col min="3" max="42" width="18.6640625" style="2" customWidth="1"/>
-    <col min="43" max="16384" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="14.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.69921875" style="2" customWidth="1"/>
+    <col min="3" max="42" width="18.69921875" style="2" customWidth="1"/>
+    <col min="43" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2870,7 +2917,7 @@
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
     </row>
-    <row r="2" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -2900,10 +2947,28 @@
       <c r="AK2" s="3"/>
       <c r="AP2" s="3"/>
     </row>
-    <row r="3" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
-      <c r="G3" s="4" t="str">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>13523155</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ref="G3:G66" si="0">IF(COUNT(C3:F3)=0,"",AVERAGE(C3:F3))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
@@ -2913,7 +2978,7 @@
       <c r="AK3" s="4"/>
       <c r="AP3" s="4"/>
     </row>
-    <row r="4" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2926,7 +2991,7 @@
       <c r="AK4" s="4"/>
       <c r="AP4" s="4"/>
     </row>
-    <row r="5" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G5" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2939,7 +3004,7 @@
       <c r="AK5" s="4"/>
       <c r="AP5" s="4"/>
     </row>
-    <row r="6" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G6" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2952,7 +3017,7 @@
       <c r="AK6" s="4"/>
       <c r="AP6" s="4"/>
     </row>
-    <row r="7" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G7" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2965,7 +3030,7 @@
       <c r="AK7" s="4"/>
       <c r="AP7" s="4"/>
     </row>
-    <row r="8" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G8" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2978,7 +3043,7 @@
       <c r="AK8" s="4"/>
       <c r="AP8" s="4"/>
     </row>
-    <row r="9" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G9" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2991,7 +3056,7 @@
       <c r="AK9" s="4"/>
       <c r="AP9" s="4"/>
     </row>
-    <row r="10" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G10" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3004,7 +3069,7 @@
       <c r="AK10" s="4"/>
       <c r="AP10" s="4"/>
     </row>
-    <row r="11" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G11" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3017,7 +3082,7 @@
       <c r="AK11" s="4"/>
       <c r="AP11" s="4"/>
     </row>
-    <row r="12" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G12" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3030,7 +3095,7 @@
       <c r="AK12" s="4"/>
       <c r="AP12" s="4"/>
     </row>
-    <row r="13" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G13" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3043,7 +3108,7 @@
       <c r="AK13" s="4"/>
       <c r="AP13" s="4"/>
     </row>
-    <row r="14" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G14" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3056,7 +3121,7 @@
       <c r="AK14" s="4"/>
       <c r="AP14" s="4"/>
     </row>
-    <row r="15" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G15" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3069,7 +3134,7 @@
       <c r="AK15" s="4"/>
       <c r="AP15" s="4"/>
     </row>
-    <row r="16" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G16" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3082,7 +3147,7 @@
       <c r="AK16" s="4"/>
       <c r="AP16" s="4"/>
     </row>
-    <row r="17" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="17" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G17" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3095,7 +3160,7 @@
       <c r="AK17" s="4"/>
       <c r="AP17" s="4"/>
     </row>
-    <row r="18" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="18" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G18" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3108,7 +3173,7 @@
       <c r="AK18" s="4"/>
       <c r="AP18" s="4"/>
     </row>
-    <row r="19" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="19" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G19" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3121,7 +3186,7 @@
       <c r="AK19" s="4"/>
       <c r="AP19" s="4"/>
     </row>
-    <row r="20" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="20" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G20" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3134,7 +3199,7 @@
       <c r="AK20" s="4"/>
       <c r="AP20" s="4"/>
     </row>
-    <row r="21" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="21" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G21" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3147,7 +3212,7 @@
       <c r="AK21" s="4"/>
       <c r="AP21" s="4"/>
     </row>
-    <row r="22" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="22" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G22" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3160,7 +3225,7 @@
       <c r="AK22" s="4"/>
       <c r="AP22" s="4"/>
     </row>
-    <row r="23" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="23" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G23" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3173,7 +3238,7 @@
       <c r="AK23" s="4"/>
       <c r="AP23" s="4"/>
     </row>
-    <row r="24" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="24" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G24" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3186,7 +3251,7 @@
       <c r="AK24" s="4"/>
       <c r="AP24" s="4"/>
     </row>
-    <row r="25" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="25" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G25" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3199,7 +3264,7 @@
       <c r="AK25" s="4"/>
       <c r="AP25" s="4"/>
     </row>
-    <row r="26" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="26" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G26" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3212,7 +3277,7 @@
       <c r="AK26" s="4"/>
       <c r="AP26" s="4"/>
     </row>
-    <row r="27" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="27" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G27" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3225,7 +3290,7 @@
       <c r="AK27" s="4"/>
       <c r="AP27" s="4"/>
     </row>
-    <row r="28" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="28" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G28" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3238,7 +3303,7 @@
       <c r="AK28" s="4"/>
       <c r="AP28" s="4"/>
     </row>
-    <row r="29" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="29" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G29" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3251,7 +3316,7 @@
       <c r="AK29" s="4"/>
       <c r="AP29" s="4"/>
     </row>
-    <row r="30" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="30" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G30" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3264,7 +3329,7 @@
       <c r="AK30" s="4"/>
       <c r="AP30" s="4"/>
     </row>
-    <row r="31" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="31" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G31" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3277,7 +3342,7 @@
       <c r="AK31" s="4"/>
       <c r="AP31" s="4"/>
     </row>
-    <row r="32" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="32" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G32" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3290,7 +3355,7 @@
       <c r="AK32" s="4"/>
       <c r="AP32" s="4"/>
     </row>
-    <row r="33" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="33" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G33" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3303,7 +3368,7 @@
       <c r="AK33" s="4"/>
       <c r="AP33" s="4"/>
     </row>
-    <row r="34" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="34" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G34" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3316,7 +3381,7 @@
       <c r="AK34" s="4"/>
       <c r="AP34" s="4"/>
     </row>
-    <row r="35" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="35" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G35" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3329,7 +3394,7 @@
       <c r="AK35" s="4"/>
       <c r="AP35" s="4"/>
     </row>
-    <row r="36" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="36" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G36" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3342,7 +3407,7 @@
       <c r="AK36" s="4"/>
       <c r="AP36" s="4"/>
     </row>
-    <row r="37" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="37" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G37" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3355,7 +3420,7 @@
       <c r="AK37" s="4"/>
       <c r="AP37" s="4"/>
     </row>
-    <row r="38" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="38" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G38" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3368,7 +3433,7 @@
       <c r="AK38" s="4"/>
       <c r="AP38" s="4"/>
     </row>
-    <row r="39" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="39" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G39" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3381,7 +3446,7 @@
       <c r="AK39" s="4"/>
       <c r="AP39" s="4"/>
     </row>
-    <row r="40" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="40" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G40" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3394,7 +3459,7 @@
       <c r="AK40" s="4"/>
       <c r="AP40" s="4"/>
     </row>
-    <row r="41" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="41" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G41" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3407,7 +3472,7 @@
       <c r="AK41" s="4"/>
       <c r="AP41" s="4"/>
     </row>
-    <row r="42" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="42" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G42" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3420,7 +3485,7 @@
       <c r="AK42" s="4"/>
       <c r="AP42" s="4"/>
     </row>
-    <row r="43" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="43" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G43" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3433,7 +3498,7 @@
       <c r="AK43" s="4"/>
       <c r="AP43" s="4"/>
     </row>
-    <row r="44" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="44" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G44" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3446,7 +3511,7 @@
       <c r="AK44" s="4"/>
       <c r="AP44" s="4"/>
     </row>
-    <row r="45" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="45" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G45" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3459,7 +3524,7 @@
       <c r="AK45" s="4"/>
       <c r="AP45" s="4"/>
     </row>
-    <row r="46" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="46" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G46" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3472,7 +3537,7 @@
       <c r="AK46" s="4"/>
       <c r="AP46" s="4"/>
     </row>
-    <row r="47" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="47" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G47" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3485,7 +3550,7 @@
       <c r="AK47" s="4"/>
       <c r="AP47" s="4"/>
     </row>
-    <row r="48" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="48" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G48" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3498,7 +3563,7 @@
       <c r="AK48" s="4"/>
       <c r="AP48" s="4"/>
     </row>
-    <row r="49" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="49" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G49" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3511,7 +3576,7 @@
       <c r="AK49" s="4"/>
       <c r="AP49" s="4"/>
     </row>
-    <row r="50" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="50" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G50" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3524,7 +3589,7 @@
       <c r="AK50" s="4"/>
       <c r="AP50" s="4"/>
     </row>
-    <row r="51" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="51" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G51" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3537,7 +3602,7 @@
       <c r="AK51" s="4"/>
       <c r="AP51" s="4"/>
     </row>
-    <row r="52" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="52" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G52" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3550,7 +3615,7 @@
       <c r="AK52" s="4"/>
       <c r="AP52" s="4"/>
     </row>
-    <row r="53" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="53" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G53" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3563,7 +3628,7 @@
       <c r="AK53" s="4"/>
       <c r="AP53" s="4"/>
     </row>
-    <row r="54" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="54" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G54" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3576,7 +3641,7 @@
       <c r="AK54" s="4"/>
       <c r="AP54" s="4"/>
     </row>
-    <row r="55" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="55" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G55" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3589,7 +3654,7 @@
       <c r="AK55" s="4"/>
       <c r="AP55" s="4"/>
     </row>
-    <row r="56" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="56" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G56" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3602,7 +3667,7 @@
       <c r="AK56" s="4"/>
       <c r="AP56" s="4"/>
     </row>
-    <row r="57" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="57" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G57" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3615,7 +3680,7 @@
       <c r="AK57" s="4"/>
       <c r="AP57" s="4"/>
     </row>
-    <row r="58" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="58" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G58" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3628,7 +3693,7 @@
       <c r="AK58" s="4"/>
       <c r="AP58" s="4"/>
     </row>
-    <row r="59" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="59" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G59" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3641,7 +3706,7 @@
       <c r="AK59" s="4"/>
       <c r="AP59" s="4"/>
     </row>
-    <row r="60" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="60" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G60" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3654,7 +3719,7 @@
       <c r="AK60" s="4"/>
       <c r="AP60" s="4"/>
     </row>
-    <row r="61" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="61" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G61" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3667,7 +3732,7 @@
       <c r="AK61" s="4"/>
       <c r="AP61" s="4"/>
     </row>
-    <row r="62" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="62" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G62" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3680,7 +3745,7 @@
       <c r="AK62" s="4"/>
       <c r="AP62" s="4"/>
     </row>
-    <row r="63" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="63" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G63" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3693,7 +3758,7 @@
       <c r="AK63" s="4"/>
       <c r="AP63" s="4"/>
     </row>
-    <row r="64" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="64" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G64" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3706,7 +3771,7 @@
       <c r="AK64" s="4"/>
       <c r="AP64" s="4"/>
     </row>
-    <row r="65" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="65" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G65" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3719,7 +3784,7 @@
       <c r="AK65" s="4"/>
       <c r="AP65" s="4"/>
     </row>
-    <row r="66" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="66" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G66" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3732,7 +3797,7 @@
       <c r="AK66" s="4"/>
       <c r="AP66" s="4"/>
     </row>
-    <row r="67" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="67" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G67" s="4" t="str">
         <f t="shared" ref="G67:G82" si="1">IF(COUNT(C67:F67)=0,"",AVERAGE(C67:F67))</f>
         <v/>
@@ -3745,7 +3810,7 @@
       <c r="AK67" s="4"/>
       <c r="AP67" s="4"/>
     </row>
-    <row r="68" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="68" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G68" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3758,7 +3823,7 @@
       <c r="AK68" s="4"/>
       <c r="AP68" s="4"/>
     </row>
-    <row r="69" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="69" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G69" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3771,7 +3836,7 @@
       <c r="AK69" s="4"/>
       <c r="AP69" s="4"/>
     </row>
-    <row r="70" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="70" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G70" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3784,7 +3849,7 @@
       <c r="AK70" s="4"/>
       <c r="AP70" s="4"/>
     </row>
-    <row r="71" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="71" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G71" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3797,7 +3862,7 @@
       <c r="AK71" s="4"/>
       <c r="AP71" s="4"/>
     </row>
-    <row r="72" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="72" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G72" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3810,7 +3875,7 @@
       <c r="AK72" s="4"/>
       <c r="AP72" s="4"/>
     </row>
-    <row r="73" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="73" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G73" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3823,7 +3888,7 @@
       <c r="AK73" s="4"/>
       <c r="AP73" s="4"/>
     </row>
-    <row r="74" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="74" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G74" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3836,7 +3901,7 @@
       <c r="AK74" s="4"/>
       <c r="AP74" s="4"/>
     </row>
-    <row r="75" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="75" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G75" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3849,7 +3914,7 @@
       <c r="AK75" s="4"/>
       <c r="AP75" s="4"/>
     </row>
-    <row r="76" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="76" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G76" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3862,7 +3927,7 @@
       <c r="AK76" s="4"/>
       <c r="AP76" s="4"/>
     </row>
-    <row r="77" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="77" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G77" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3875,7 +3940,7 @@
       <c r="AK77" s="4"/>
       <c r="AP77" s="4"/>
     </row>
-    <row r="78" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="78" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G78" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3888,7 +3953,7 @@
       <c r="AK78" s="4"/>
       <c r="AP78" s="4"/>
     </row>
-    <row r="79" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="79" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G79" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3901,7 +3966,7 @@
       <c r="AK79" s="4"/>
       <c r="AP79" s="4"/>
     </row>
-    <row r="80" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="80" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G80" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3914,7 +3979,7 @@
       <c r="AK80" s="4"/>
       <c r="AP80" s="4"/>
     </row>
-    <row r="81" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="81" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G81" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3927,7 +3992,7 @@
       <c r="AK81" s="4"/>
       <c r="AP81" s="4"/>
     </row>
-    <row r="82" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="82" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G82" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3954,15 +4019,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50D1F948-1ADF-4B33-979B-06CD398BC5BF}">
   <dimension ref="A1:AP82"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="2" customWidth="1"/>
-    <col min="3" max="42" width="18.6640625" style="2" customWidth="1"/>
-    <col min="43" max="16384" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="14.69921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.69921875" style="2" customWidth="1"/>
+    <col min="3" max="42" width="18.69921875" style="2" customWidth="1"/>
+    <col min="43" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4020,7 +4085,7 @@
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
     </row>
-    <row r="2" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -4050,10 +4115,28 @@
       <c r="AK2" s="3"/>
       <c r="AP2" s="3"/>
     </row>
-    <row r="3" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
-      <c r="G3" s="4" t="str">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>13523155</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ref="G3:G66" si="0">IF(COUNT(C3:F3)=0,"",AVERAGE(C3:F3))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="L3" s="4"/>
       <c r="Q3" s="4"/>
@@ -4063,7 +4146,7 @@
       <c r="AK3" s="4"/>
       <c r="AP3" s="4"/>
     </row>
-    <row r="4" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G4" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4076,7 +4159,7 @@
       <c r="AK4" s="4"/>
       <c r="AP4" s="4"/>
     </row>
-    <row r="5" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G5" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4089,7 +4172,7 @@
       <c r="AK5" s="4"/>
       <c r="AP5" s="4"/>
     </row>
-    <row r="6" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G6" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4102,7 +4185,7 @@
       <c r="AK6" s="4"/>
       <c r="AP6" s="4"/>
     </row>
-    <row r="7" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G7" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4115,7 +4198,7 @@
       <c r="AK7" s="4"/>
       <c r="AP7" s="4"/>
     </row>
-    <row r="8" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G8" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4128,7 +4211,7 @@
       <c r="AK8" s="4"/>
       <c r="AP8" s="4"/>
     </row>
-    <row r="9" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G9" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4141,7 +4224,7 @@
       <c r="AK9" s="4"/>
       <c r="AP9" s="4"/>
     </row>
-    <row r="10" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G10" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4154,7 +4237,7 @@
       <c r="AK10" s="4"/>
       <c r="AP10" s="4"/>
     </row>
-    <row r="11" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G11" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4167,7 +4250,7 @@
       <c r="AK11" s="4"/>
       <c r="AP11" s="4"/>
     </row>
-    <row r="12" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G12" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4180,7 +4263,7 @@
       <c r="AK12" s="4"/>
       <c r="AP12" s="4"/>
     </row>
-    <row r="13" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G13" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4193,7 +4276,7 @@
       <c r="AK13" s="4"/>
       <c r="AP13" s="4"/>
     </row>
-    <row r="14" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G14" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4206,7 +4289,7 @@
       <c r="AK14" s="4"/>
       <c r="AP14" s="4"/>
     </row>
-    <row r="15" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G15" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4219,7 +4302,7 @@
       <c r="AK15" s="4"/>
       <c r="AP15" s="4"/>
     </row>
-    <row r="16" spans="1:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.3">
       <c r="G16" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4232,7 +4315,7 @@
       <c r="AK16" s="4"/>
       <c r="AP16" s="4"/>
     </row>
-    <row r="17" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="17" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G17" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4245,7 +4328,7 @@
       <c r="AK17" s="4"/>
       <c r="AP17" s="4"/>
     </row>
-    <row r="18" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="18" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G18" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4258,7 +4341,7 @@
       <c r="AK18" s="4"/>
       <c r="AP18" s="4"/>
     </row>
-    <row r="19" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="19" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G19" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4271,7 +4354,7 @@
       <c r="AK19" s="4"/>
       <c r="AP19" s="4"/>
     </row>
-    <row r="20" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="20" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G20" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4284,7 +4367,7 @@
       <c r="AK20" s="4"/>
       <c r="AP20" s="4"/>
     </row>
-    <row r="21" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="21" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G21" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4297,7 +4380,7 @@
       <c r="AK21" s="4"/>
       <c r="AP21" s="4"/>
     </row>
-    <row r="22" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="22" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G22" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4310,7 +4393,7 @@
       <c r="AK22" s="4"/>
       <c r="AP22" s="4"/>
     </row>
-    <row r="23" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="23" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G23" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4323,7 +4406,7 @@
       <c r="AK23" s="4"/>
       <c r="AP23" s="4"/>
     </row>
-    <row r="24" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="24" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G24" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4336,7 +4419,7 @@
       <c r="AK24" s="4"/>
       <c r="AP24" s="4"/>
     </row>
-    <row r="25" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="25" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G25" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4349,7 +4432,7 @@
       <c r="AK25" s="4"/>
       <c r="AP25" s="4"/>
     </row>
-    <row r="26" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="26" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G26" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4362,7 +4445,7 @@
       <c r="AK26" s="4"/>
       <c r="AP26" s="4"/>
     </row>
-    <row r="27" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="27" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G27" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4375,7 +4458,7 @@
       <c r="AK27" s="4"/>
       <c r="AP27" s="4"/>
     </row>
-    <row r="28" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="28" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G28" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4388,7 +4471,7 @@
       <c r="AK28" s="4"/>
       <c r="AP28" s="4"/>
     </row>
-    <row r="29" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="29" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G29" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4401,7 +4484,7 @@
       <c r="AK29" s="4"/>
       <c r="AP29" s="4"/>
     </row>
-    <row r="30" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="30" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G30" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4414,7 +4497,7 @@
       <c r="AK30" s="4"/>
       <c r="AP30" s="4"/>
     </row>
-    <row r="31" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="31" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G31" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4427,7 +4510,7 @@
       <c r="AK31" s="4"/>
       <c r="AP31" s="4"/>
     </row>
-    <row r="32" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="32" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G32" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4440,7 +4523,7 @@
       <c r="AK32" s="4"/>
       <c r="AP32" s="4"/>
     </row>
-    <row r="33" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="33" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G33" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4453,7 +4536,7 @@
       <c r="AK33" s="4"/>
       <c r="AP33" s="4"/>
     </row>
-    <row r="34" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="34" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G34" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4466,7 +4549,7 @@
       <c r="AK34" s="4"/>
       <c r="AP34" s="4"/>
     </row>
-    <row r="35" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="35" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G35" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4479,7 +4562,7 @@
       <c r="AK35" s="4"/>
       <c r="AP35" s="4"/>
     </row>
-    <row r="36" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="36" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G36" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4492,7 +4575,7 @@
       <c r="AK36" s="4"/>
       <c r="AP36" s="4"/>
     </row>
-    <row r="37" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="37" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G37" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4505,7 +4588,7 @@
       <c r="AK37" s="4"/>
       <c r="AP37" s="4"/>
     </row>
-    <row r="38" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="38" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G38" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4518,7 +4601,7 @@
       <c r="AK38" s="4"/>
       <c r="AP38" s="4"/>
     </row>
-    <row r="39" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="39" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G39" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4531,7 +4614,7 @@
       <c r="AK39" s="4"/>
       <c r="AP39" s="4"/>
     </row>
-    <row r="40" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="40" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G40" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4544,7 +4627,7 @@
       <c r="AK40" s="4"/>
       <c r="AP40" s="4"/>
     </row>
-    <row r="41" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="41" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G41" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4557,7 +4640,7 @@
       <c r="AK41" s="4"/>
       <c r="AP41" s="4"/>
     </row>
-    <row r="42" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="42" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G42" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4570,7 +4653,7 @@
       <c r="AK42" s="4"/>
       <c r="AP42" s="4"/>
     </row>
-    <row r="43" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="43" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G43" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4583,7 +4666,7 @@
       <c r="AK43" s="4"/>
       <c r="AP43" s="4"/>
     </row>
-    <row r="44" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="44" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G44" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4596,7 +4679,7 @@
       <c r="AK44" s="4"/>
       <c r="AP44" s="4"/>
     </row>
-    <row r="45" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="45" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G45" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4609,7 +4692,7 @@
       <c r="AK45" s="4"/>
       <c r="AP45" s="4"/>
     </row>
-    <row r="46" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="46" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G46" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4622,7 +4705,7 @@
       <c r="AK46" s="4"/>
       <c r="AP46" s="4"/>
     </row>
-    <row r="47" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="47" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G47" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4635,7 +4718,7 @@
       <c r="AK47" s="4"/>
       <c r="AP47" s="4"/>
     </row>
-    <row r="48" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="48" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G48" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4648,7 +4731,7 @@
       <c r="AK48" s="4"/>
       <c r="AP48" s="4"/>
     </row>
-    <row r="49" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="49" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G49" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4661,7 +4744,7 @@
       <c r="AK49" s="4"/>
       <c r="AP49" s="4"/>
     </row>
-    <row r="50" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="50" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G50" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4674,7 +4757,7 @@
       <c r="AK50" s="4"/>
       <c r="AP50" s="4"/>
     </row>
-    <row r="51" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="51" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G51" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4687,7 +4770,7 @@
       <c r="AK51" s="4"/>
       <c r="AP51" s="4"/>
     </row>
-    <row r="52" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="52" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G52" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4700,7 +4783,7 @@
       <c r="AK52" s="4"/>
       <c r="AP52" s="4"/>
     </row>
-    <row r="53" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="53" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G53" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4713,7 +4796,7 @@
       <c r="AK53" s="4"/>
       <c r="AP53" s="4"/>
     </row>
-    <row r="54" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="54" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G54" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4726,7 +4809,7 @@
       <c r="AK54" s="4"/>
       <c r="AP54" s="4"/>
     </row>
-    <row r="55" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="55" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G55" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4739,7 +4822,7 @@
       <c r="AK55" s="4"/>
       <c r="AP55" s="4"/>
     </row>
-    <row r="56" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="56" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G56" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4752,7 +4835,7 @@
       <c r="AK56" s="4"/>
       <c r="AP56" s="4"/>
     </row>
-    <row r="57" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="57" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G57" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4765,7 +4848,7 @@
       <c r="AK57" s="4"/>
       <c r="AP57" s="4"/>
     </row>
-    <row r="58" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="58" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G58" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4778,7 +4861,7 @@
       <c r="AK58" s="4"/>
       <c r="AP58" s="4"/>
     </row>
-    <row r="59" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="59" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G59" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4791,7 +4874,7 @@
       <c r="AK59" s="4"/>
       <c r="AP59" s="4"/>
     </row>
-    <row r="60" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="60" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G60" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4804,7 +4887,7 @@
       <c r="AK60" s="4"/>
       <c r="AP60" s="4"/>
     </row>
-    <row r="61" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="61" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G61" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4817,7 +4900,7 @@
       <c r="AK61" s="4"/>
       <c r="AP61" s="4"/>
     </row>
-    <row r="62" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="62" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G62" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4830,7 +4913,7 @@
       <c r="AK62" s="4"/>
       <c r="AP62" s="4"/>
     </row>
-    <row r="63" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="63" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G63" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4843,7 +4926,7 @@
       <c r="AK63" s="4"/>
       <c r="AP63" s="4"/>
     </row>
-    <row r="64" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="64" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G64" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4856,7 +4939,7 @@
       <c r="AK64" s="4"/>
       <c r="AP64" s="4"/>
     </row>
-    <row r="65" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="65" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G65" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4869,7 +4952,7 @@
       <c r="AK65" s="4"/>
       <c r="AP65" s="4"/>
     </row>
-    <row r="66" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="66" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G66" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4882,7 +4965,7 @@
       <c r="AK66" s="4"/>
       <c r="AP66" s="4"/>
     </row>
-    <row r="67" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="67" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G67" s="4" t="str">
         <f t="shared" ref="G67:G82" si="1">IF(COUNT(C67:F67)=0,"",AVERAGE(C67:F67))</f>
         <v/>
@@ -4895,7 +4978,7 @@
       <c r="AK67" s="4"/>
       <c r="AP67" s="4"/>
     </row>
-    <row r="68" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="68" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G68" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4908,7 +4991,7 @@
       <c r="AK68" s="4"/>
       <c r="AP68" s="4"/>
     </row>
-    <row r="69" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="69" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G69" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4921,7 +5004,7 @@
       <c r="AK69" s="4"/>
       <c r="AP69" s="4"/>
     </row>
-    <row r="70" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="70" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G70" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4934,7 +5017,7 @@
       <c r="AK70" s="4"/>
       <c r="AP70" s="4"/>
     </row>
-    <row r="71" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="71" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G71" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4947,7 +5030,7 @@
       <c r="AK71" s="4"/>
       <c r="AP71" s="4"/>
     </row>
-    <row r="72" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="72" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G72" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4960,7 +5043,7 @@
       <c r="AK72" s="4"/>
       <c r="AP72" s="4"/>
     </row>
-    <row r="73" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="73" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G73" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4973,7 +5056,7 @@
       <c r="AK73" s="4"/>
       <c r="AP73" s="4"/>
     </row>
-    <row r="74" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="74" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G74" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4986,7 +5069,7 @@
       <c r="AK74" s="4"/>
       <c r="AP74" s="4"/>
     </row>
-    <row r="75" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="75" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G75" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4999,7 +5082,7 @@
       <c r="AK75" s="4"/>
       <c r="AP75" s="4"/>
     </row>
-    <row r="76" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="76" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G76" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5012,7 +5095,7 @@
       <c r="AK76" s="4"/>
       <c r="AP76" s="4"/>
     </row>
-    <row r="77" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="77" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G77" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5025,7 +5108,7 @@
       <c r="AK77" s="4"/>
       <c r="AP77" s="4"/>
     </row>
-    <row r="78" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="78" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G78" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5038,7 +5121,7 @@
       <c r="AK78" s="4"/>
       <c r="AP78" s="4"/>
     </row>
-    <row r="79" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="79" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G79" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5051,7 +5134,7 @@
       <c r="AK79" s="4"/>
       <c r="AP79" s="4"/>
     </row>
-    <row r="80" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="80" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G80" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5064,7 +5147,7 @@
       <c r="AK80" s="4"/>
       <c r="AP80" s="4"/>
     </row>
-    <row r="81" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="81" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G81" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5077,7 +5160,7 @@
       <c r="AK81" s="4"/>
       <c r="AP81" s="4"/>
     </row>
-    <row r="82" spans="7:42" ht="14.75" x14ac:dyDescent="0.75">
+    <row r="82" spans="7:42" x14ac:dyDescent="0.3">
       <c r="G82" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>

</xml_diff>